<commit_message>
Types de logement : Studio/T2/T3/T4 partout (au lieu de 'Appartement')
CONVENTION (validée 2026-04-28)
- Studio : maisonnette, apolove, miniloveroom, grandeloveroom, kingston
- T2 (1 chambre + séjour) : kitesurf, hamac, paddle, surf, cocon, facemer, grandlarge, albatros, JEANNE (Cœur de Berck), evasion
- T3 (2 chambres + séjour) : balneo, apollo, terrasse, rotonde, patio
- T4 (3 chambres + séjour) : famille
- À préciser : reserve

JEANNE = T2 (Cœur de Berck) — confirmé par Claudine

Mise à jour dans :
- index.html APPART_INFO (typeLogement)
- trello-data/build-recap-excel-utf8.ps1 (type)
- recap-apparts.xlsx régénéré
</commit_message>
<xml_diff>
--- a/recap-apparts.xlsx
+++ b/recap-apparts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\claud\Downloads\livret-accueil\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BC141054-03CF-46B9-AB67-FBE6211A378B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BABE4093-89E5-4408-96BE-DE9E0098790E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19298" yWindow="-2415" windowWidth="19396" windowHeight="11475" xr2:uid="{C2AF825C-61BD-43DD-825D-E784788557D2}"/>
+    <workbookView xWindow="-19298" yWindow="-2415" windowWidth="19396" windowHeight="11475" xr2:uid="{C7E3364C-1F3B-4F82-B69D-FE4C602E3587}"/>
   </bookViews>
   <sheets>
     <sheet name="Récap 22 apparts" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="913" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="913" uniqueCount="243">
   <si>
     <t>#</t>
   </si>
@@ -177,418 +177,421 @@
     <t>marechal</t>
   </si>
   <si>
+    <t>T2</t>
+  </si>
+  <si>
+    <t>34 m²</t>
+  </si>
+  <si>
+    <t>4 couchages · chambre 160×200 · canapé gigogne 2×(90×190)</t>
+  </si>
+  <si>
+    <t>2e étage</t>
+  </si>
+  <si>
+    <t>Non</t>
+  </si>
+  <si>
+    <t>Dans la rue</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1yoVLVnDSSuuU90lgiMc3-EHvn3vVVqLv/view</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=HVP1-x_L478</t>
+  </si>
+  <si>
+    <t>Vitro-céramique</t>
+  </si>
+  <si>
+    <t>Compartiment freezer</t>
+  </si>
+  <si>
+    <t>Senseo + filtre</t>
+  </si>
+  <si>
+    <t>Oui</t>
+  </si>
+  <si>
+    <t>Oui (assiettes, verres, casserole, poêle, plat à tarte)</t>
+  </si>
+  <si>
+    <t>Oui (hypoallergénique, OK enfants)</t>
+  </si>
+  <si>
+    <t>Molotov standard</t>
+  </si>
+  <si>
+    <t>BBOX - 4929C743</t>
+  </si>
+  <si>
+    <t>KXv9 DNH2 uDd5 n165 1u</t>
+  </si>
+  <si>
+    <t>Non (en option)</t>
+  </si>
+  <si>
+    <t>Oui (sur demande)</t>
+  </si>
+  <si>
+    <t>Rémi</t>
+  </si>
+  <si>
+    <t>LMP</t>
+  </si>
+  <si>
+    <t>hamac</t>
+  </si>
+  <si>
+    <t>Hamac</t>
+  </si>
+  <si>
+    <t>35 m²</t>
+  </si>
+  <si>
+    <t>4 couchages · chambre 160×200 · canapé convertible 140×190</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1FsKU-XGly3eeHe0fYpDQ3sFK3GM3jpBg/view</t>
+  </si>
+  <si>
+    <t>BBOX-4DA61D</t>
+  </si>
+  <si>
+    <t>9LMRXwLjC3qRxMLU93</t>
+  </si>
+  <si>
+    <t>Non (lit double + canapé-lit)</t>
+  </si>
+  <si>
+    <t>paddle</t>
+  </si>
+  <si>
+    <t>Paddle</t>
+  </si>
+  <si>
+    <t>30 m²</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1lRwnNiII1xYEauzS5ddg6J4jKLQm9uum/view</t>
+  </si>
+  <si>
+    <t>BBOX-39A25D</t>
+  </si>
+  <si>
+    <t>Twuy7AjqMpFAY3bSTM</t>
+  </si>
+  <si>
+    <t>surf</t>
+  </si>
+  <si>
+    <t>Surf</t>
+  </si>
+  <si>
+    <t>1er étage</t>
+  </si>
+  <si>
+    <t>BBOX-1A4DA8</t>
+  </si>
+  <si>
+    <t>To check</t>
+  </si>
+  <si>
+    <t>famille</t>
+  </si>
+  <si>
+    <t>Famille</t>
+  </si>
+  <si>
+    <t>3 Chambres 100m Plage</t>
+  </si>
+  <si>
+    <t>T4</t>
+  </si>
+  <si>
+    <t>70 m²</t>
+  </si>
+  <si>
+    <t>6+ couchages · 3 chambres</t>
+  </si>
+  <si>
+    <t>À préciser</t>
+  </si>
+  <si>
+    <t>Induction</t>
+  </si>
+  <si>
+    <t>Frigo + congélateur séparé</t>
+  </si>
+  <si>
+    <t>Famille-Berck</t>
+  </si>
+  <si>
+    <t>balneo</t>
+  </si>
+  <si>
+    <t>Balnéo</t>
+  </si>
+  <si>
+    <t>Balnéo Garden</t>
+  </si>
+  <si>
+    <t>25 rue Maréchal Juin, 62600 Berck</t>
+  </si>
+  <si>
+    <t>Le 25</t>
+  </si>
+  <si>
+    <t>T3</t>
+  </si>
+  <si>
+    <t>53 m²</t>
+  </si>
+  <si>
+    <t>6 couchages · chambre 1: 160×200 · chambre 2: 2×(90×190) · canapé 140×190</t>
+  </si>
+  <si>
+    <t>RDC</t>
+  </si>
+  <si>
+    <t>✅ Parking sécurisé inclus</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1tc8QjWR0X3tYzfez82oHtJ4DMdQ2uLhw/view</t>
+  </si>
+  <si>
+    <t>Frigo américain (congélateur intégré)</t>
+  </si>
+  <si>
+    <t>Cetana (2 places face à face)</t>
+  </si>
+  <si>
+    <t>BBOX-CE0F6E</t>
+  </si>
+  <si>
+    <t>Clara</t>
+  </si>
+  <si>
+    <t>cocon</t>
+  </si>
+  <si>
+    <t>Cocon Romantique</t>
+  </si>
+  <si>
+    <t>40 m²</t>
+  </si>
+  <si>
+    <t>2 couchages · chambre 160×200</t>
+  </si>
+  <si>
+    <t>Cocon-Berck</t>
+  </si>
+  <si>
+    <t>terrasse</t>
+  </si>
+  <si>
+    <t>Terrasse</t>
+  </si>
+  <si>
+    <t>La Terrasse</t>
+  </si>
+  <si>
+    <t>17 rue du Grand Hôtel, 62600 Berck</t>
+  </si>
+  <si>
+    <t>63 m²</t>
+  </si>
+  <si>
+    <t>8 couchages · chambre 1: 160×200 · chambre 2: 140×200 + 2×(90×190) · canapé 140×190</t>
+  </si>
+  <si>
+    <t>Terrasse-Berck</t>
+  </si>
+  <si>
+    <t>✅ Lit bébé + chaise haute</t>
+  </si>
+  <si>
+    <t>Christelle</t>
+  </si>
+  <si>
+    <t>maisonnette</t>
+  </si>
+  <si>
+    <t>Maisonnette</t>
+  </si>
+  <si>
+    <t>Cœur des Sables</t>
+  </si>
+  <si>
+    <t>2 rue des Sables, 62600 Berck</t>
+  </si>
+  <si>
+    <t>Studio</t>
+  </si>
+  <si>
+    <t>23 m²</t>
+  </si>
+  <si>
+    <t>2 lits · 160×200</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/14nBlb8KgwoHIzeLN7z8mi9n9eAP6CuAq/view</t>
+  </si>
+  <si>
+    <t>Senseo</t>
+  </si>
+  <si>
+    <t>Maisonnette-Berck</t>
+  </si>
+  <si>
+    <t>facemer</t>
+  </si>
+  <si>
+    <t>Face Mer</t>
+  </si>
+  <si>
+    <t>Face Mer Esplanade</t>
+  </si>
+  <si>
+    <t>1 rue de la Plage, 62600 Berck</t>
+  </si>
+  <si>
+    <t>esplanade</t>
+  </si>
+  <si>
+    <t>Oui (vue mer)</t>
+  </si>
+  <si>
+    <t>FaceMer-Berck</t>
+  </si>
+  <si>
+    <t>grandlarge</t>
+  </si>
+  <si>
+    <t>Grand Large</t>
+  </si>
+  <si>
+    <t>Hamac Face Mer</t>
+  </si>
+  <si>
+    <t>45 Esplanade Parmentier, 62600 Berck</t>
+  </si>
+  <si>
+    <t>38 m²</t>
+  </si>
+  <si>
+    <t>3e étage</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1yT8uTNvdaBE5eM7y-VJIBBW5zskDZLfD/view</t>
+  </si>
+  <si>
+    <t>Oui (hamac)</t>
+  </si>
+  <si>
+    <t>GrandLarge-Berck</t>
+  </si>
+  <si>
+    <t>SAS Maréchal Invest</t>
+  </si>
+  <si>
+    <t>apolove</t>
+  </si>
+  <si>
+    <t>Apolove</t>
+  </si>
+  <si>
+    <t>Suite Romantique Face Mer</t>
+  </si>
+  <si>
+    <t>2 Avenue Marianne (studio), 62600 Berck</t>
+  </si>
+  <si>
+    <t>Apollo</t>
+  </si>
+  <si>
+    <t>25 m²</t>
+  </si>
+  <si>
+    <t>5e étage</t>
+  </si>
+  <si>
+    <t>✅ Parking couvert n°206 inclus (résidence Albatros, rue Saint-Louis)</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1AFgKVhahrxvljkL7vVa8ZU1-zA0BgHwo/view</t>
+  </si>
+  <si>
+    <t>Indra Wave (compact, 2 personnes face à face)</t>
+  </si>
+  <si>
+    <t>suite2</t>
+  </si>
+  <si>
+    <t>2Avmarianne</t>
+  </si>
+  <si>
+    <t>❌ Interdits</t>
+  </si>
+  <si>
+    <t>apollo</t>
+  </si>
+  <si>
+    <t>Panoramique 2 Chambres</t>
+  </si>
+  <si>
+    <t>2 Avenue Marianne (T3), 62600 Berck</t>
+  </si>
+  <si>
+    <t>6 couchages · 2 chambres 160×200 · canapé 140×190</t>
+  </si>
+  <si>
+    <t>✅ Parking n°502 inclus (portail avec bip)</t>
+  </si>
+  <si>
+    <t>Oui (vue panoramique)</t>
+  </si>
+  <si>
+    <t>Apollo-Berck</t>
+  </si>
+  <si>
+    <t>kingston</t>
+  </si>
+  <si>
+    <t>Kingston</t>
+  </si>
+  <si>
+    <t>Face Mer Exceptionnel</t>
+  </si>
+  <si>
+    <t>2 Avenue Marianne (appt 16, RDC), 62600 Berck</t>
+  </si>
+  <si>
+    <t>47 m²</t>
+  </si>
+  <si>
+    <t>4 couchages · canapé lit 160</t>
+  </si>
+  <si>
+    <t>✅ Parking n°16 inclus (juste devant)</t>
+  </si>
+  <si>
+    <t>Kingston-Berck</t>
+  </si>
+  <si>
+    <t>SCI</t>
+  </si>
+  <si>
+    <t>reserve</t>
+  </si>
+  <si>
+    <t>La Réserve</t>
+  </si>
+  <si>
+    <t>2 Avenue Marianne, 62600 Berck</t>
+  </si>
+  <si>
     <t>Appartement</t>
-  </si>
-  <si>
-    <t>34 m²</t>
-  </si>
-  <si>
-    <t>4 couchages · chambre 160×200 · canapé gigogne 2×(90×190)</t>
-  </si>
-  <si>
-    <t>2e étage</t>
-  </si>
-  <si>
-    <t>Non</t>
-  </si>
-  <si>
-    <t>Dans la rue</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1yoVLVnDSSuuU90lgiMc3-EHvn3vVVqLv/view</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=HVP1-x_L478</t>
-  </si>
-  <si>
-    <t>Vitro-céramique</t>
-  </si>
-  <si>
-    <t>Compartiment freezer</t>
-  </si>
-  <si>
-    <t>Senseo + filtre</t>
-  </si>
-  <si>
-    <t>Oui</t>
-  </si>
-  <si>
-    <t>Oui (assiettes, verres, casserole, poêle, plat à tarte)</t>
-  </si>
-  <si>
-    <t>Oui (hypoallergénique, OK enfants)</t>
-  </si>
-  <si>
-    <t>Molotov standard</t>
-  </si>
-  <si>
-    <t>BBOX - 4929C743</t>
-  </si>
-  <si>
-    <t>KXv9 DNH2 uDd5 n165 1u</t>
-  </si>
-  <si>
-    <t>Non (en option)</t>
-  </si>
-  <si>
-    <t>Oui (sur demande)</t>
-  </si>
-  <si>
-    <t>Rémi</t>
-  </si>
-  <si>
-    <t>LMP</t>
-  </si>
-  <si>
-    <t>hamac</t>
-  </si>
-  <si>
-    <t>Hamac</t>
-  </si>
-  <si>
-    <t>35 m²</t>
-  </si>
-  <si>
-    <t>4 couchages · chambre 160×200 · canapé convertible 140×190</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1FsKU-XGly3eeHe0fYpDQ3sFK3GM3jpBg/view</t>
-  </si>
-  <si>
-    <t>BBOX-4DA61D</t>
-  </si>
-  <si>
-    <t>9LMRXwLjC3qRxMLU93</t>
-  </si>
-  <si>
-    <t>Non (lit double + canapé-lit)</t>
-  </si>
-  <si>
-    <t>paddle</t>
-  </si>
-  <si>
-    <t>Paddle</t>
-  </si>
-  <si>
-    <t>30 m²</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1lRwnNiII1xYEauzS5ddg6J4jKLQm9uum/view</t>
-  </si>
-  <si>
-    <t>BBOX-39A25D</t>
-  </si>
-  <si>
-    <t>Twuy7AjqMpFAY3bSTM</t>
-  </si>
-  <si>
-    <t>surf</t>
-  </si>
-  <si>
-    <t>Surf</t>
-  </si>
-  <si>
-    <t>1er étage</t>
-  </si>
-  <si>
-    <t>BBOX-1A4DA8</t>
-  </si>
-  <si>
-    <t>To check</t>
-  </si>
-  <si>
-    <t>famille</t>
-  </si>
-  <si>
-    <t>Famille</t>
-  </si>
-  <si>
-    <t>3 Chambres 100m Plage</t>
-  </si>
-  <si>
-    <t>Grand appartement 3 chambres</t>
-  </si>
-  <si>
-    <t>70 m²</t>
-  </si>
-  <si>
-    <t>6+ couchages · 3 chambres</t>
-  </si>
-  <si>
-    <t>À préciser</t>
-  </si>
-  <si>
-    <t>Induction</t>
-  </si>
-  <si>
-    <t>Frigo + congélateur séparé</t>
-  </si>
-  <si>
-    <t>Famille-Berck</t>
-  </si>
-  <si>
-    <t>balneo</t>
-  </si>
-  <si>
-    <t>Balnéo</t>
-  </si>
-  <si>
-    <t>Balnéo Garden</t>
-  </si>
-  <si>
-    <t>25 rue Maréchal Juin, 62600 Berck</t>
-  </si>
-  <si>
-    <t>Le 25</t>
-  </si>
-  <si>
-    <t>53 m²</t>
-  </si>
-  <si>
-    <t>6 couchages · chambre 1: 160×200 · chambre 2: 2×(90×190) · canapé 140×190</t>
-  </si>
-  <si>
-    <t>RDC</t>
-  </si>
-  <si>
-    <t>✅ Parking sécurisé inclus</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1tc8QjWR0X3tYzfez82oHtJ4DMdQ2uLhw/view</t>
-  </si>
-  <si>
-    <t>Frigo américain (congélateur intégré)</t>
-  </si>
-  <si>
-    <t>Cetana (2 places face à face)</t>
-  </si>
-  <si>
-    <t>BBOX-CE0F6E</t>
-  </si>
-  <si>
-    <t>Clara</t>
-  </si>
-  <si>
-    <t>cocon</t>
-  </si>
-  <si>
-    <t>Cocon Romantique</t>
-  </si>
-  <si>
-    <t>40 m²</t>
-  </si>
-  <si>
-    <t>2 couchages · chambre 160×200</t>
-  </si>
-  <si>
-    <t>Cocon-Berck</t>
-  </si>
-  <si>
-    <t>terrasse</t>
-  </si>
-  <si>
-    <t>Terrasse</t>
-  </si>
-  <si>
-    <t>La Terrasse</t>
-  </si>
-  <si>
-    <t>17 rue du Grand Hôtel, 62600 Berck</t>
-  </si>
-  <si>
-    <t>Grand appartement</t>
-  </si>
-  <si>
-    <t>63 m²</t>
-  </si>
-  <si>
-    <t>8 couchages · chambre 1: 160×200 · chambre 2: 140×200 + 2×(90×190) · canapé 140×190</t>
-  </si>
-  <si>
-    <t>Terrasse-Berck</t>
-  </si>
-  <si>
-    <t>✅ Lit bébé + chaise haute</t>
-  </si>
-  <si>
-    <t>Christelle</t>
-  </si>
-  <si>
-    <t>maisonnette</t>
-  </si>
-  <si>
-    <t>Maisonnette</t>
-  </si>
-  <si>
-    <t>Cœur des Sables</t>
-  </si>
-  <si>
-    <t>2 rue des Sables, 62600 Berck</t>
-  </si>
-  <si>
-    <t>Studio</t>
-  </si>
-  <si>
-    <t>23 m²</t>
-  </si>
-  <si>
-    <t>2 lits · 160×200</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/14nBlb8KgwoHIzeLN7z8mi9n9eAP6CuAq/view</t>
-  </si>
-  <si>
-    <t>Senseo</t>
-  </si>
-  <si>
-    <t>Maisonnette-Berck</t>
-  </si>
-  <si>
-    <t>facemer</t>
-  </si>
-  <si>
-    <t>Face Mer</t>
-  </si>
-  <si>
-    <t>Face Mer Esplanade</t>
-  </si>
-  <si>
-    <t>1 rue de la Plage, 62600 Berck</t>
-  </si>
-  <si>
-    <t>esplanade</t>
-  </si>
-  <si>
-    <t>Oui (vue mer)</t>
-  </si>
-  <si>
-    <t>FaceMer-Berck</t>
-  </si>
-  <si>
-    <t>grandlarge</t>
-  </si>
-  <si>
-    <t>Grand Large</t>
-  </si>
-  <si>
-    <t>Hamac Face Mer</t>
-  </si>
-  <si>
-    <t>45 Esplanade Parmentier, 62600 Berck</t>
-  </si>
-  <si>
-    <t>38 m²</t>
-  </si>
-  <si>
-    <t>3e étage</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1yT8uTNvdaBE5eM7y-VJIBBW5zskDZLfD/view</t>
-  </si>
-  <si>
-    <t>Oui (hamac)</t>
-  </si>
-  <si>
-    <t>GrandLarge-Berck</t>
-  </si>
-  <si>
-    <t>SAS Maréchal Invest</t>
-  </si>
-  <si>
-    <t>apolove</t>
-  </si>
-  <si>
-    <t>Apolove</t>
-  </si>
-  <si>
-    <t>Suite Romantique Face Mer</t>
-  </si>
-  <si>
-    <t>2 Avenue Marianne (studio), 62600 Berck</t>
-  </si>
-  <si>
-    <t>Apollo</t>
-  </si>
-  <si>
-    <t>25 m²</t>
-  </si>
-  <si>
-    <t>5e étage</t>
-  </si>
-  <si>
-    <t>✅ Parking couvert n°206 inclus (résidence Albatros, rue Saint-Louis)</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/file/d/1AFgKVhahrxvljkL7vVa8ZU1-zA0BgHwo/view</t>
-  </si>
-  <si>
-    <t>Indra Wave (compact, 2 personnes face à face)</t>
-  </si>
-  <si>
-    <t>suite2</t>
-  </si>
-  <si>
-    <t>2Avmarianne</t>
-  </si>
-  <si>
-    <t>❌ Interdits</t>
-  </si>
-  <si>
-    <t>apollo</t>
-  </si>
-  <si>
-    <t>Panoramique 2 Chambres</t>
-  </si>
-  <si>
-    <t>2 Avenue Marianne (T3), 62600 Berck</t>
-  </si>
-  <si>
-    <t>6 couchages · 2 chambres 160×200 · canapé 140×190</t>
-  </si>
-  <si>
-    <t>✅ Parking n°502 inclus (portail avec bip)</t>
-  </si>
-  <si>
-    <t>Oui (vue panoramique)</t>
-  </si>
-  <si>
-    <t>Apollo-Berck</t>
-  </si>
-  <si>
-    <t>kingston</t>
-  </si>
-  <si>
-    <t>Kingston</t>
-  </si>
-  <si>
-    <t>Face Mer Exceptionnel</t>
-  </si>
-  <si>
-    <t>2 Avenue Marianne (appt 16, RDC), 62600 Berck</t>
-  </si>
-  <si>
-    <t>47 m²</t>
-  </si>
-  <si>
-    <t>4 couchages · canapé lit 160</t>
-  </si>
-  <si>
-    <t>✅ Parking n°16 inclus (juste devant)</t>
-  </si>
-  <si>
-    <t>Kingston-Berck</t>
-  </si>
-  <si>
-    <t>SCI</t>
-  </si>
-  <si>
-    <t>reserve</t>
-  </si>
-  <si>
-    <t>La Réserve</t>
-  </si>
-  <si>
-    <t>2 Avenue Marianne, 62600 Berck</t>
   </si>
   <si>
     <t>albatros</t>
@@ -1124,7 +1127,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{288E1F18-D171-4377-95E7-0C47466054CE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC4FF69D-7B54-43FC-8A35-2F58943C80CA}">
   <dimension ref="A1:AR23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1134,7 +1137,7 @@
     <col min="4" max="4" width="23.81640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="35.6328125" customWidth="1"/>
     <col min="6" max="7" width="12.6328125" customWidth="1"/>
-    <col min="8" max="8" width="27.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.26953125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.6328125" customWidth="1"/>
     <col min="10" max="10" width="35.6328125" customWidth="1"/>
     <col min="11" max="11" width="22.54296875" bestFit="1" customWidth="1"/>
@@ -1988,25 +1991,25 @@
         <v>48</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>49</v>
+        <v>104</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>53</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="O7" s="2" t="s">
         <v>56</v>
@@ -2015,7 +2018,7 @@
         <v>57</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="R7" s="2" t="s">
         <v>59</v>
@@ -2045,7 +2048,7 @@
         <v>60</v>
       </c>
       <c r="AA7" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AB7" s="2" t="s">
         <v>53</v>
@@ -2066,7 +2069,7 @@
         <v>1</v>
       </c>
       <c r="AH7" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="AI7" s="2" t="s">
         <v>88</v>
@@ -2090,7 +2093,7 @@
         <v>53</v>
       </c>
       <c r="AP7" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AQ7" s="2" t="s">
         <v>69</v>
@@ -2104,13 +2107,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>102</v>
@@ -2125,13 +2128,13 @@
         <v>49</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>53</v>
@@ -2177,7 +2180,7 @@
         <v>60</v>
       </c>
       <c r="AA8" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AB8" s="2" t="s">
         <v>60</v>
@@ -2198,7 +2201,7 @@
         <v>1</v>
       </c>
       <c r="AH8" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AI8" s="2" t="s">
         <v>88</v>
@@ -2222,7 +2225,7 @@
         <v>53</v>
       </c>
       <c r="AP8" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AQ8" s="2" t="s">
         <v>69</v>
@@ -2236,25 +2239,25 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>118</v>
-      </c>
       <c r="H9" s="2" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>123</v>
@@ -2263,7 +2266,7 @@
         <v>124</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>53</v>
@@ -2380,10 +2383,10 @@
         <v>131</v>
       </c>
       <c r="F10" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>132</v>
@@ -2395,7 +2398,7 @@
         <v>134</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>53</v>
@@ -2792,7 +2795,7 @@
         <v>160</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>161</v>
@@ -2888,7 +2891,7 @@
         <v>53</v>
       </c>
       <c r="AP13" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AQ13" s="2" t="s">
         <v>154</v>
@@ -2920,10 +2923,10 @@
         <v>142</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>49</v>
+        <v>104</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>171</v>
@@ -2945,7 +2948,7 @@
         <v>57</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="R14" s="2" t="s">
         <v>59</v>
@@ -3020,7 +3023,7 @@
         <v>53</v>
       </c>
       <c r="AP14" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AQ14" s="2" t="s">
         <v>154</v>
@@ -3052,7 +3055,7 @@
         <v>142</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>49</v>
+        <v>132</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>179</v>
@@ -3061,7 +3064,7 @@
         <v>180</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>53</v>
@@ -3152,7 +3155,7 @@
         <v>53</v>
       </c>
       <c r="AP15" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AQ15" s="2" t="s">
         <v>183</v>
@@ -3184,7 +3187,7 @@
         <v>142</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>49</v>
+        <v>187</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>95</v>
@@ -3284,7 +3287,7 @@
         <v>53</v>
       </c>
       <c r="AP16" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AQ16" s="2" t="s">
         <v>154</v>
@@ -3298,19 +3301,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D17" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>189</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>188</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>142</v>
@@ -3322,7 +3325,7 @@
         <v>160</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>150</v>
@@ -3334,7 +3337,7 @@
         <v>54</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="O17" s="2" t="s">
         <v>56</v>
@@ -3379,7 +3382,7 @@
         <v>53</v>
       </c>
       <c r="AC17" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="AD17" s="2" t="s">
         <v>53</v>
@@ -3394,7 +3397,7 @@
         <v>1</v>
       </c>
       <c r="AH17" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AI17" s="2" t="s">
         <v>88</v>
@@ -3418,7 +3421,7 @@
         <v>53</v>
       </c>
       <c r="AP17" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AQ17" s="2" t="s">
         <v>154</v>
@@ -3432,19 +3435,19 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>142</v>
@@ -3453,10 +3456,10 @@
         <v>132</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="K18" s="2" t="s">
         <v>150</v>
@@ -3468,7 +3471,7 @@
         <v>54</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="O18" s="2" t="s">
         <v>56</v>
@@ -3477,7 +3480,7 @@
         <v>57</v>
       </c>
       <c r="Q18" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="R18" s="2" t="s">
         <v>136</v>
@@ -3522,13 +3525,13 @@
         <v>53</v>
       </c>
       <c r="AF18" s="2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AG18" s="2">
         <v>1</v>
       </c>
       <c r="AH18" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI18" s="2" t="s">
         <v>88</v>
@@ -3566,19 +3569,19 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>142</v>
@@ -3587,10 +3590,10 @@
         <v>132</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="K19" s="2" t="s">
         <v>150</v>
@@ -3660,7 +3663,7 @@
         <v>1</v>
       </c>
       <c r="AH19" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="AI19" s="2" t="s">
         <v>88</v>
@@ -3698,49 +3701,49 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C20" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>212</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>211</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>49</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="L20" s="2" t="s">
         <v>53</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="O20" s="2" t="s">
         <v>56</v>
       </c>
       <c r="P20" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="Q20" s="2" t="s">
         <v>97</v>
@@ -3794,7 +3797,7 @@
         <v>1</v>
       </c>
       <c r="AH20" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AI20" s="2">
         <v>83968280</v>
@@ -3832,22 +3835,22 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>49</v>
@@ -3856,7 +3859,7 @@
         <v>149</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K21" s="2" t="s">
         <v>86</v>
@@ -3865,10 +3868,10 @@
         <v>53</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="O21" s="2" t="s">
         <v>56</v>
@@ -3907,7 +3910,7 @@
         <v>60</v>
       </c>
       <c r="AA21" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AB21" s="2" t="s">
         <v>60</v>
@@ -3928,7 +3931,7 @@
         <v>1</v>
       </c>
       <c r="AH21" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="AI21" s="2" t="s">
         <v>88</v>
@@ -3966,40 +3969,40 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>49</v>
+        <v>104</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="L22" s="2" t="s">
         <v>53</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2" t="s">
@@ -4039,10 +4042,10 @@
         <v>60</v>
       </c>
       <c r="AA22" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AB22" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AC22" s="2" t="s">
         <v>53</v>
@@ -4060,7 +4063,7 @@
         <v>1</v>
       </c>
       <c r="AH22" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="AI22" s="2" t="s">
         <v>88</v>
@@ -4098,43 +4101,43 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>49</v>
+        <v>187</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>179</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="L23" s="2" t="s">
         <v>53</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="O23" s="2" t="s">
         <v>56</v>
@@ -4173,13 +4176,13 @@
         <v>60</v>
       </c>
       <c r="AA23" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AB23" s="2" t="s">
         <v>53</v>
       </c>
       <c r="AC23" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="AD23" s="2" t="s">
         <v>60</v>
@@ -4194,7 +4197,7 @@
         <v>1</v>
       </c>
       <c r="AH23" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AI23" s="2" t="s">
         <v>88</v>
@@ -4228,7 +4231,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AR23" xr:uid="{288E1F18-D171-4377-95E7-0C47466054CE}"/>
+  <autoFilter ref="A1:AR23" xr:uid="{AC4FF69D-7B54-43FC-8A35-2F58943C80CA}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Excel récap : couleurs (vert=Oui, rose=Non, orange=À préciser) pour lecture rapide
</commit_message>
<xml_diff>
--- a/recap-apparts.xlsx
+++ b/recap-apparts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\claud\Downloads\livret-accueil\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BABE4093-89E5-4408-96BE-DE9E0098790E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{73C2A44B-BA5E-4A1A-8254-02C40151DE18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19298" yWindow="-2415" windowWidth="19396" windowHeight="11475" xr2:uid="{C7E3364C-1F3B-4F82-B69D-FE4C602E3587}"/>
+    <workbookView xWindow="-19298" yWindow="-2415" windowWidth="19396" windowHeight="11475" xr2:uid="{F23E13F6-63B1-41C1-9CD1-9E56B1B168B4}"/>
   </bookViews>
   <sheets>
     <sheet name="Récap 22 apparts" sheetId="1" r:id="rId1"/>
@@ -780,7 +780,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -790,6 +790,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF101510"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC8C8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC9E6C8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE0B8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -806,12 +824,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1127,7 +1154,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC4FF69D-7B54-43FC-8A35-2F58943C80CA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A64D7D0E-AB10-4B85-8329-05C462C9F18A}">
   <dimension ref="A1:AR23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1336,7 +1363,7 @@
       <c r="K2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M2" s="2" t="s">
@@ -1357,43 +1384,43 @@
       <c r="R2" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U2" s="2" t="s">
+      <c r="S2" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T2" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U2" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V2" s="2" t="s">
+      <c r="V2" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AD2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE2" s="2" t="s">
+      <c r="W2" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X2" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y2" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z2" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA2" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB2" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC2" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD2" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE2" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF2" s="2" t="s">
@@ -1411,19 +1438,19 @@
       <c r="AJ2" s="2">
         <v>15</v>
       </c>
-      <c r="AK2" s="2" t="s">
+      <c r="AK2" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="AL2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM2" s="2" t="s">
+      <c r="AL2" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM2" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO2" s="2" t="s">
+      <c r="AN2" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO2" s="4" t="s">
         <v>60</v>
       </c>
       <c r="AP2" s="2" t="s">
@@ -1470,7 +1497,7 @@
       <c r="K3" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L3" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M3" s="2" t="s">
@@ -1491,43 +1518,43 @@
       <c r="R3" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S3" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U3" s="2" t="s">
+      <c r="S3" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U3" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V3" s="2" t="s">
+      <c r="V3" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W3" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X3" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y3" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z3" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA3" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB3" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC3" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AD3" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE3" s="2" t="s">
+      <c r="W3" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X3" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z3" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC3" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE3" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF3" s="2" t="s">
@@ -1545,19 +1572,19 @@
       <c r="AJ3" s="2">
         <v>15</v>
       </c>
-      <c r="AK3" s="2" t="s">
+      <c r="AK3" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="AL3" s="2" t="s">
+      <c r="AL3" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="AM3" s="2" t="s">
+      <c r="AM3" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN3" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO3" s="2" t="s">
+      <c r="AN3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO3" s="4" t="s">
         <v>60</v>
       </c>
       <c r="AP3" s="2" t="s">
@@ -1604,7 +1631,7 @@
       <c r="K4" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="L4" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M4" s="2" t="s">
@@ -1625,43 +1652,43 @@
       <c r="R4" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S4" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T4" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U4" s="2" t="s">
+      <c r="S4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U4" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V4" s="2" t="s">
+      <c r="V4" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W4" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X4" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y4" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z4" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA4" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB4" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC4" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AD4" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE4" s="2" t="s">
+      <c r="W4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE4" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF4" s="2" t="s">
@@ -1679,19 +1706,19 @@
       <c r="AJ4" s="2">
         <v>15</v>
       </c>
-      <c r="AK4" s="2" t="s">
+      <c r="AK4" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="AL4" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM4" s="2" t="s">
+      <c r="AL4" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM4" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN4" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO4" s="2" t="s">
+      <c r="AN4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO4" s="4" t="s">
         <v>60</v>
       </c>
       <c r="AP4" s="2" t="s">
@@ -1738,7 +1765,7 @@
       <c r="K5" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="L5" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M5" s="2" t="s">
@@ -1757,43 +1784,43 @@
       <c r="R5" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S5" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T5" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U5" s="2" t="s">
+      <c r="S5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U5" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V5" s="2" t="s">
+      <c r="V5" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W5" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X5" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y5" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z5" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA5" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB5" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC5" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AD5" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE5" s="2" t="s">
+      <c r="W5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y5" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA5" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB5" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD5" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE5" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF5" s="2" t="s">
@@ -1811,19 +1838,19 @@
       <c r="AJ5" s="2">
         <v>15</v>
       </c>
-      <c r="AK5" s="2" t="s">
+      <c r="AK5" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="AL5" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM5" s="2" t="s">
+      <c r="AL5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM5" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN5" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO5" s="2" t="s">
+      <c r="AN5" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO5" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP5" s="2" t="s">
@@ -1867,10 +1894,10 @@
       <c r="J6" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="K6" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="L6" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M6" s="2" t="s">
@@ -1889,43 +1916,43 @@
       <c r="R6" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S6" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T6" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U6" s="2" t="s">
+      <c r="S6" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T6" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U6" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V6" s="2" t="s">
+      <c r="V6" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W6" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X6" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y6" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z6" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA6" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB6" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC6" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AD6" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE6" s="2" t="s">
+      <c r="W6" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X6" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z6" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE6" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF6" s="2" t="s">
@@ -1943,19 +1970,19 @@
       <c r="AJ6" s="2">
         <v>15</v>
       </c>
-      <c r="AK6" s="2" t="s">
+      <c r="AK6" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="AL6" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM6" s="2" t="s">
+      <c r="AL6" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM6" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN6" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO6" s="2" t="s">
+      <c r="AN6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO6" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP6" s="2" t="s">
@@ -2002,7 +2029,7 @@
       <c r="K7" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="L7" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M7" s="2" t="s">
@@ -2023,43 +2050,43 @@
       <c r="R7" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S7" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T7" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U7" s="2" t="s">
+      <c r="S7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U7" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V7" s="2" t="s">
+      <c r="V7" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W7" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X7" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y7" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z7" s="2" t="s">
+      <c r="W7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z7" s="4" t="s">
         <v>60</v>
       </c>
       <c r="AA7" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="AB7" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC7" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AD7" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AE7" s="2" t="s">
+      <c r="AB7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE7" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF7" s="2" t="s">
@@ -2077,19 +2104,19 @@
       <c r="AJ7" s="2">
         <v>20</v>
       </c>
-      <c r="AK7" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL7" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM7" s="2" t="s">
+      <c r="AK7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM7" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN7" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO7" s="2" t="s">
+      <c r="AN7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO7" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP7" s="2" t="s">
@@ -2136,7 +2163,7 @@
       <c r="K8" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="L8" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M8" s="2" t="s">
@@ -2155,43 +2182,43 @@
       <c r="R8" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U8" s="2" t="s">
+      <c r="S8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U8" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V8" s="2" t="s">
+      <c r="V8" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z8" s="2" t="s">
+      <c r="W8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z8" s="4" t="s">
         <v>60</v>
       </c>
       <c r="AA8" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="AB8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AC8" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AD8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AE8" s="2" t="s">
+      <c r="AB8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AC8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE8" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF8" s="2" t="s">
@@ -2209,19 +2236,19 @@
       <c r="AJ8" s="2">
         <v>20</v>
       </c>
-      <c r="AK8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM8" s="2" t="s">
+      <c r="AK8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM8" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN8" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO8" s="2" t="s">
+      <c r="AN8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO8" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP8" s="2" t="s">
@@ -2268,7 +2295,7 @@
       <c r="K9" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="L9" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M9" s="2" t="s">
@@ -2287,43 +2314,43 @@
       <c r="R9" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S9" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T9" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U9" s="2" t="s">
+      <c r="S9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U9" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V9" s="2" t="s">
+      <c r="V9" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W9" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X9" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y9" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z9" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA9" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB9" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC9" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AD9" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE9" s="2" t="s">
+      <c r="W9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE9" s="4" t="s">
         <v>60</v>
       </c>
       <c r="AF9" s="2" t="s">
@@ -2341,19 +2368,19 @@
       <c r="AJ9" s="2">
         <v>15</v>
       </c>
-      <c r="AK9" s="2" t="s">
+      <c r="AK9" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="AL9" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM9" s="2" t="s">
+      <c r="AL9" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM9" s="4" t="s">
         <v>67</v>
       </c>
       <c r="AN9" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="AO9" s="2" t="s">
+      <c r="AO9" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP9" s="2" t="s">
@@ -2400,7 +2427,7 @@
       <c r="K10" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="L10" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M10" s="2" t="s">
@@ -2421,43 +2448,43 @@
       <c r="R10" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="S10" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T10" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U10" s="2" t="s">
+      <c r="S10" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T10" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U10" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V10" s="2" t="s">
+      <c r="V10" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W10" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X10" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Y10" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z10" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA10" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB10" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC10" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AD10" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AE10" s="2" t="s">
+      <c r="W10" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Y10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z10" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC10" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD10" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE10" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF10" s="2" t="s">
@@ -2475,19 +2502,19 @@
       <c r="AJ10" s="2">
         <v>15</v>
       </c>
-      <c r="AK10" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL10" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM10" s="2" t="s">
+      <c r="AK10" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL10" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM10" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN10" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO10" s="2" t="s">
+      <c r="AN10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO10" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP10" s="2" t="s">
@@ -2525,16 +2552,16 @@
       <c r="H11" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="J11" s="5" t="s">
         <v>95</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="L11" s="2" t="s">
+      <c r="L11" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M11" s="2" t="s">
@@ -2553,43 +2580,43 @@
       <c r="R11" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S11" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T11" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U11" s="2" t="s">
+      <c r="S11" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T11" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U11" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V11" s="2" t="s">
+      <c r="V11" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W11" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X11" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y11" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z11" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA11" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB11" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC11" s="2" t="s">
+      <c r="W11" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X11" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y11" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z11" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA11" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB11" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC11" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="AD11" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE11" s="2" t="s">
+      <c r="AD11" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE11" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF11" s="2" t="s">
@@ -2607,19 +2634,19 @@
       <c r="AJ11" s="2">
         <v>15</v>
       </c>
-      <c r="AK11" s="2" t="s">
+      <c r="AK11" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="AL11" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM11" s="2" t="s">
+      <c r="AL11" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM11" s="4" t="s">
         <v>67</v>
       </c>
       <c r="AN11" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="AO11" s="2" t="s">
+      <c r="AO11" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP11" s="2" t="s">
@@ -2666,7 +2693,7 @@
       <c r="K12" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="L12" s="2" t="s">
+      <c r="L12" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M12" s="2" t="s">
@@ -2687,43 +2714,43 @@
       <c r="R12" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S12" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T12" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U12" s="2" t="s">
+      <c r="S12" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T12" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U12" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V12" s="2" t="s">
+      <c r="V12" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W12" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X12" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y12" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z12" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA12" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB12" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC12" s="2" t="s">
+      <c r="W12" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X12" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y12" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z12" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA12" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB12" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC12" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="AD12" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE12" s="2" t="s">
+      <c r="AD12" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE12" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF12" s="2" t="s">
@@ -2741,19 +2768,19 @@
       <c r="AJ12" s="2">
         <v>15</v>
       </c>
-      <c r="AK12" s="2" t="s">
+      <c r="AK12" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="AL12" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM12" s="2" t="s">
+      <c r="AL12" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM12" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN12" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO12" s="2" t="s">
+      <c r="AN12" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO12" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP12" s="2" t="s">
@@ -2800,7 +2827,7 @@
       <c r="K13" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="L13" s="2" t="s">
+      <c r="L13" s="4" t="s">
         <v>60</v>
       </c>
       <c r="M13" s="2" t="s">
@@ -2821,43 +2848,43 @@
       <c r="R13" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S13" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T13" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U13" s="2" t="s">
+      <c r="S13" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T13" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U13" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V13" s="2" t="s">
+      <c r="V13" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W13" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="X13" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y13" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z13" s="2" t="s">
+      <c r="W13" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="X13" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y13" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z13" s="4" t="s">
         <v>60</v>
       </c>
       <c r="AA13" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="AB13" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC13" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AD13" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE13" s="2" t="s">
+      <c r="AB13" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC13" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD13" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE13" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF13" s="2" t="s">
@@ -2875,19 +2902,19 @@
       <c r="AJ13" s="2">
         <v>20</v>
       </c>
-      <c r="AK13" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL13" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM13" s="2" t="s">
+      <c r="AK13" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL13" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM13" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="AN13" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO13" s="2" t="s">
+      <c r="AN13" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO13" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP13" s="2" t="s">
@@ -2934,7 +2961,7 @@
       <c r="K14" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="L14" s="2" t="s">
+      <c r="L14" s="4" t="s">
         <v>60</v>
       </c>
       <c r="M14" s="2" t="s">
@@ -2953,43 +2980,43 @@
       <c r="R14" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S14" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T14" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U14" s="2" t="s">
+      <c r="S14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U14" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V14" s="2" t="s">
+      <c r="V14" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W14" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X14" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y14" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z14" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA14" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB14" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC14" s="2" t="s">
+      <c r="W14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC14" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="AD14" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE14" s="2" t="s">
+      <c r="AD14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE14" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF14" s="2" t="s">
@@ -3007,19 +3034,19 @@
       <c r="AJ14" s="2">
         <v>20</v>
       </c>
-      <c r="AK14" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL14" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM14" s="2" t="s">
+      <c r="AK14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM14" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="AN14" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO14" s="2" t="s">
+      <c r="AN14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO14" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP14" s="2" t="s">
@@ -3066,7 +3093,7 @@
       <c r="K15" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="L15" s="2" t="s">
+      <c r="L15" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M15" s="2" t="s">
@@ -3085,43 +3112,43 @@
       <c r="R15" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="S15" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T15" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U15" s="2" t="s">
+      <c r="S15" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T15" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U15" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V15" s="2" t="s">
+      <c r="V15" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W15" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X15" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Y15" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z15" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AA15" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB15" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC15" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AD15" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE15" s="2" t="s">
+      <c r="W15" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X15" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Y15" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z15" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AA15" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB15" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC15" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AD15" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE15" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF15" s="2" t="s">
@@ -3139,19 +3166,19 @@
       <c r="AJ15" s="2">
         <v>20</v>
       </c>
-      <c r="AK15" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL15" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM15" s="2" t="s">
+      <c r="AK15" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL15" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM15" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN15" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO15" s="2" t="s">
+      <c r="AN15" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO15" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP15" s="2" t="s">
@@ -3189,19 +3216,19 @@
       <c r="H16" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="I16" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="J16" s="2" t="s">
+      <c r="J16" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="K16" s="2" t="s">
+      <c r="K16" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="L16" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="M16" s="2" t="s">
+      <c r="L16" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="M16" s="5" t="s">
         <v>95</v>
       </c>
       <c r="N16" s="2"/>
@@ -3217,43 +3244,43 @@
       <c r="R16" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S16" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T16" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U16" s="2" t="s">
+      <c r="S16" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T16" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U16" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V16" s="2" t="s">
+      <c r="V16" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W16" s="2" t="s">
+      <c r="W16" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="X16" s="2" t="s">
+      <c r="X16" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="Y16" s="2" t="s">
+      <c r="Y16" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="Z16" s="2" t="s">
+      <c r="Z16" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="AA16" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB16" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC16" s="2" t="s">
+      <c r="AA16" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB16" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC16" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="AD16" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE16" s="2" t="s">
+      <c r="AD16" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE16" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF16" s="2" t="s">
@@ -3262,28 +3289,28 @@
       <c r="AG16" s="2">
         <v>1</v>
       </c>
-      <c r="AH16" s="2" t="s">
+      <c r="AH16" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="AI16" s="2" t="s">
+      <c r="AI16" s="5" t="s">
         <v>95</v>
       </c>
       <c r="AJ16" s="2">
         <v>20</v>
       </c>
-      <c r="AK16" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL16" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM16" s="2" t="s">
+      <c r="AK16" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL16" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM16" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN16" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO16" s="2" t="s">
+      <c r="AN16" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO16" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP16" s="2" t="s">
@@ -3330,7 +3357,7 @@
       <c r="K17" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="L17" s="2" t="s">
+      <c r="L17" s="4" t="s">
         <v>60</v>
       </c>
       <c r="M17" s="2" t="s">
@@ -3351,43 +3378,43 @@
       <c r="R17" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S17" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T17" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U17" s="2" t="s">
+      <c r="S17" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T17" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U17" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V17" s="2" t="s">
+      <c r="V17" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W17" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X17" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y17" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z17" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA17" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB17" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC17" s="2" t="s">
+      <c r="W17" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X17" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y17" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z17" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA17" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB17" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC17" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="AD17" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE17" s="2" t="s">
+      <c r="AD17" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE17" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF17" s="2" t="s">
@@ -3405,19 +3432,19 @@
       <c r="AJ17" s="2">
         <v>15</v>
       </c>
-      <c r="AK17" s="2" t="s">
+      <c r="AK17" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="AL17" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM17" s="2" t="s">
+      <c r="AL17" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM17" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN17" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO17" s="2" t="s">
+      <c r="AN17" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO17" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP17" s="2" t="s">
@@ -3464,7 +3491,7 @@
       <c r="K18" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="L18" s="2" t="s">
+      <c r="L18" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M18" s="2" t="s">
@@ -3485,43 +3512,43 @@
       <c r="R18" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="S18" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T18" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U18" s="2" t="s">
+      <c r="S18" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T18" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U18" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V18" s="2" t="s">
+      <c r="V18" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W18" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="X18" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Y18" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z18" s="2" t="s">
+      <c r="W18" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="X18" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Y18" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z18" s="4" t="s">
         <v>60</v>
       </c>
       <c r="AA18" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="AB18" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC18" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AD18" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE18" s="2" t="s">
+      <c r="AB18" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC18" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD18" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE18" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF18" s="2" t="s">
@@ -3539,19 +3566,19 @@
       <c r="AJ18" s="2">
         <v>20</v>
       </c>
-      <c r="AK18" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL18" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM18" s="2" t="s">
+      <c r="AK18" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL18" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM18" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN18" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO18" s="2" t="s">
+      <c r="AN18" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO18" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP18" s="2" t="s">
@@ -3598,7 +3625,7 @@
       <c r="K19" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="L19" s="2" t="s">
+      <c r="L19" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M19" s="2" t="s">
@@ -3617,43 +3644,43 @@
       <c r="R19" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="S19" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T19" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U19" s="2" t="s">
+      <c r="S19" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T19" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U19" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V19" s="2" t="s">
+      <c r="V19" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W19" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="X19" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y19" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z19" s="2" t="s">
+      <c r="W19" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="X19" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y19" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z19" s="4" t="s">
         <v>60</v>
       </c>
       <c r="AA19" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="AB19" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC19" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AD19" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE19" s="2" t="s">
+      <c r="AB19" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC19" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD19" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE19" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF19" s="2" t="s">
@@ -3671,19 +3698,19 @@
       <c r="AJ19" s="2">
         <v>20</v>
       </c>
-      <c r="AK19" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL19" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM19" s="2" t="s">
+      <c r="AK19" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL19" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM19" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="AN19" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO19" s="2" t="s">
+      <c r="AN19" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO19" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP19" s="2" t="s">
@@ -3730,7 +3757,7 @@
       <c r="K20" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="L20" s="2" t="s">
+      <c r="L20" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M20" s="2" t="s">
@@ -3751,43 +3778,43 @@
       <c r="R20" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S20" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T20" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U20" s="2" t="s">
+      <c r="S20" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T20" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U20" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V20" s="2" t="s">
+      <c r="V20" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W20" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X20" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Y20" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="Z20" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AA20" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB20" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC20" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AD20" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE20" s="2" t="s">
+      <c r="W20" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Y20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z20" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE20" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF20" s="2" t="s">
@@ -3805,19 +3832,19 @@
       <c r="AJ20" s="2">
         <v>15</v>
       </c>
-      <c r="AK20" s="2" t="s">
+      <c r="AK20" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="AL20" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM20" s="2" t="s">
+      <c r="AL20" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM20" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN20" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO20" s="2" t="s">
+      <c r="AN20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO20" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP20" s="2" t="s">
@@ -3864,7 +3891,7 @@
       <c r="K21" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="L21" s="2" t="s">
+      <c r="L21" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M21" s="2" t="s">
@@ -3885,43 +3912,43 @@
       <c r="R21" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S21" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T21" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U21" s="2" t="s">
+      <c r="S21" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T21" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U21" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V21" s="2" t="s">
+      <c r="V21" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W21" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X21" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y21" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z21" s="2" t="s">
+      <c r="W21" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X21" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y21" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z21" s="4" t="s">
         <v>60</v>
       </c>
       <c r="AA21" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="AB21" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AC21" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AD21" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE21" s="2" t="s">
+      <c r="AB21" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AC21" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD21" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE21" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF21" s="2" t="s">
@@ -3939,19 +3966,19 @@
       <c r="AJ21" s="2">
         <v>20</v>
       </c>
-      <c r="AK21" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL21" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM21" s="2" t="s">
+      <c r="AK21" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL21" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM21" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN21" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO21" s="2" t="s">
+      <c r="AN21" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO21" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP21" s="2" t="s">
@@ -3998,7 +4025,7 @@
       <c r="K22" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="L22" s="2" t="s">
+      <c r="L22" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M22" s="2" t="s">
@@ -4017,43 +4044,43 @@
       <c r="R22" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S22" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T22" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U22" s="2" t="s">
+      <c r="S22" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T22" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U22" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V22" s="2" t="s">
+      <c r="V22" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W22" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X22" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y22" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z22" s="2" t="s">
+      <c r="W22" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X22" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y22" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z22" s="4" t="s">
         <v>60</v>
       </c>
       <c r="AA22" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="AB22" s="2" t="s">
+      <c r="AB22" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="AC22" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AD22" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE22" s="2" t="s">
+      <c r="AC22" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AD22" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE22" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF22" s="2" t="s">
@@ -4071,19 +4098,19 @@
       <c r="AJ22" s="2">
         <v>20</v>
       </c>
-      <c r="AK22" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL22" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM22" s="2" t="s">
+      <c r="AK22" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL22" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM22" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN22" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO22" s="2" t="s">
+      <c r="AN22" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO22" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP22" s="2" t="s">
@@ -4130,7 +4157,7 @@
       <c r="K23" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="L23" s="2" t="s">
+      <c r="L23" s="3" t="s">
         <v>53</v>
       </c>
       <c r="M23" s="2" t="s">
@@ -4151,43 +4178,43 @@
       <c r="R23" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="S23" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="T23" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="U23" s="2" t="s">
+      <c r="S23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="T23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="U23" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="V23" s="2" t="s">
+      <c r="V23" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="W23" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="X23" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y23" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z23" s="2" t="s">
+      <c r="W23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="X23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Y23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z23" s="4" t="s">
         <v>60</v>
       </c>
       <c r="AA23" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="AB23" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AC23" s="2" t="s">
+      <c r="AB23" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AC23" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="AD23" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AE23" s="2" t="s">
+      <c r="AD23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AE23" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AF23" s="2" t="s">
@@ -4205,19 +4232,19 @@
       <c r="AJ23" s="2">
         <v>20</v>
       </c>
-      <c r="AK23" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AL23" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="AM23" s="2" t="s">
+      <c r="AK23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AL23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="AM23" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="AN23" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO23" s="2" t="s">
+      <c r="AN23" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO23" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AP23" s="2" t="s">
@@ -4231,7 +4258,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AR23" xr:uid="{AC4FF69D-7B54-43FC-8A35-2F58943C80CA}"/>
+  <autoFilter ref="A1:AR23" xr:uid="{A64D7D0E-AB10-4B85-8329-05C462C9F18A}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
WiFi : SSID/mots de passe complets dans l'Excel + Jeanne/Évasion = TV antenne hertzienne (pas Molotov)
WIFI EXCEL — corrections à partir du livret HTML (source de vérité)
- hamac : TP LINK E2E4 / 40803500
- surf : SURF / Marechal
- balneo + cocon : XXX_63B8 / 89tnbr3bqk33pwkp8tjj
- terrasse : xxxx_5ACO / qpvr6qkj76bhcb6uyw25
- facemer : SFR_39E8 / facemercentreesplanade
- grandlarge : TP link D1EE / 74817733
- apollo : TP link DODO / 15246653
- kingston : TP-LINK -B2A5 / 82562328
- albatros : TP link D1E8 / 66436003
- mini + grande love room : Romance / 58Facemer
- evasion + jeanne : TP-LINK _6322 / 83968280
- rotonde + patio : Patio23 / 23Patio23
- (famille + reserve : À préciser)

TV ANTENNE — Jeanne + Évasion
- Pas de Molotov dans ces 2 apparts (antenne hertzienne TNT classique)
- Nouvelle carte 'Télévision — Antenne hertzienne' dans le guide pratique
- Excel : tv='Antenne hertzienne (TNT)'
</commit_message>
<xml_diff>
--- a/recap-apparts.xlsx
+++ b/recap-apparts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\claud\Downloads\livret-accueil\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{73C2A44B-BA5E-4A1A-8254-02C40151DE18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C955FC4B-EDD6-4679-A0A9-9345A56E12D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19298" yWindow="-2415" windowWidth="19396" windowHeight="11475" xr2:uid="{F23E13F6-63B1-41C1-9CD1-9E56B1B168B4}"/>
+    <workbookView xWindow="-19298" yWindow="-2415" windowWidth="19396" windowHeight="11475" xr2:uid="{97D192CB-F2F3-47CF-8BF7-D87EE467ED9C}"/>
   </bookViews>
   <sheets>
     <sheet name="Récap 22 apparts" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="913" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="243">
   <si>
     <t>#</t>
   </si>
@@ -255,10 +255,7 @@
     <t>https://drive.google.com/file/d/1FsKU-XGly3eeHe0fYpDQ3sFK3GM3jpBg/view</t>
   </si>
   <si>
-    <t>BBOX-4DA61D</t>
-  </si>
-  <si>
-    <t>9LMRXwLjC3qRxMLU93</t>
+    <t>TP LINK E2E4</t>
   </si>
   <si>
     <t>Non (lit double + canapé-lit)</t>
@@ -276,12 +273,6 @@
     <t>https://drive.google.com/file/d/1lRwnNiII1xYEauzS5ddg6J4jKLQm9uum/view</t>
   </si>
   <si>
-    <t>BBOX-39A25D</t>
-  </si>
-  <si>
-    <t>Twuy7AjqMpFAY3bSTM</t>
-  </si>
-  <si>
     <t>surf</t>
   </si>
   <si>
@@ -291,42 +282,45 @@
     <t>1er étage</t>
   </si>
   <si>
-    <t>BBOX-1A4DA8</t>
+    <t>SURF</t>
+  </si>
+  <si>
+    <t>Marechal</t>
+  </si>
+  <si>
+    <t>famille</t>
+  </si>
+  <si>
+    <t>Famille</t>
+  </si>
+  <si>
+    <t>3 Chambres 100m Plage</t>
+  </si>
+  <si>
+    <t>T4</t>
+  </si>
+  <si>
+    <t>70 m²</t>
+  </si>
+  <si>
+    <t>6+ couchages · 3 chambres</t>
+  </si>
+  <si>
+    <t>À préciser</t>
+  </si>
+  <si>
+    <t>Induction</t>
+  </si>
+  <si>
+    <t>Frigo + congélateur séparé</t>
+  </si>
+  <si>
+    <t>A préciser</t>
   </si>
   <si>
     <t>To check</t>
   </si>
   <si>
-    <t>famille</t>
-  </si>
-  <si>
-    <t>Famille</t>
-  </si>
-  <si>
-    <t>3 Chambres 100m Plage</t>
-  </si>
-  <si>
-    <t>T4</t>
-  </si>
-  <si>
-    <t>70 m²</t>
-  </si>
-  <si>
-    <t>6+ couchages · 3 chambres</t>
-  </si>
-  <si>
-    <t>À préciser</t>
-  </si>
-  <si>
-    <t>Induction</t>
-  </si>
-  <si>
-    <t>Frigo + congélateur séparé</t>
-  </si>
-  <si>
-    <t>Famille-Berck</t>
-  </si>
-  <si>
     <t>balneo</t>
   </si>
   <si>
@@ -366,7 +360,10 @@
     <t>Cetana (2 places face à face)</t>
   </si>
   <si>
-    <t>BBOX-CE0F6E</t>
+    <t>XXX_63B8</t>
+  </si>
+  <si>
+    <t>89tnbr3bqk33pwkp8tjj</t>
   </si>
   <si>
     <t>Clara</t>
@@ -384,9 +381,6 @@
     <t>2 couchages · chambre 160×200</t>
   </si>
   <si>
-    <t>Cocon-Berck</t>
-  </si>
-  <si>
     <t>terrasse</t>
   </si>
   <si>
@@ -405,7 +399,10 @@
     <t>8 couchages · chambre 1: 160×200 · chambre 2: 140×200 + 2×(90×190) · canapé 140×190</t>
   </si>
   <si>
-    <t>Terrasse-Berck</t>
+    <t>xxxx_5ACO</t>
+  </si>
+  <si>
+    <t>qpvr6qkj76bhcb6uyw25</t>
   </si>
   <si>
     <t>✅ Lit bébé + chaise haute</t>
@@ -462,7 +459,10 @@
     <t>Oui (vue mer)</t>
   </si>
   <si>
-    <t>FaceMer-Berck</t>
+    <t>SFR_39E8</t>
+  </si>
+  <si>
+    <t>facemercentreesplanade</t>
   </si>
   <si>
     <t>grandlarge</t>
@@ -489,7 +489,7 @@
     <t>Oui (hamac)</t>
   </si>
   <si>
-    <t>GrandLarge-Berck</t>
+    <t>TP link D1EE</t>
   </si>
   <si>
     <t>SAS Maréchal Invest</t>
@@ -552,7 +552,7 @@
     <t>Oui (vue panoramique)</t>
   </si>
   <si>
-    <t>Apollo-Berck</t>
+    <t>TP link DODO</t>
   </si>
   <si>
     <t>kingston</t>
@@ -576,7 +576,7 @@
     <t>✅ Parking n°16 inclus (juste devant)</t>
   </si>
   <si>
-    <t>Kingston-Berck</t>
+    <t>TP-LINK -B2A5</t>
   </si>
   <si>
     <t>SCI</t>
@@ -615,7 +615,7 @@
     <t>Non (local à vélos)</t>
   </si>
   <si>
-    <t>Albatros-Berck</t>
+    <t>TP link D1E8</t>
   </si>
   <si>
     <t>miniloveroom</t>
@@ -648,7 +648,10 @@
     <t>Vidéoprojecteur + Molotov Premium</t>
   </si>
   <si>
-    <t>MiniLove-Berck</t>
+    <t>Romance</t>
+  </si>
+  <si>
+    <t>58Facemer</t>
   </si>
   <si>
     <t>grandeloveroom</t>
@@ -663,9 +666,6 @@
     <t>28 m²</t>
   </si>
   <si>
-    <t>GrandeLove-Berck</t>
-  </si>
-  <si>
     <t>jeanne</t>
   </si>
   <si>
@@ -699,6 +699,9 @@
     <t>Gaz</t>
   </si>
   <si>
+    <t>Antenne hertzienne (TNT)</t>
+  </si>
+  <si>
     <t>TP-LINK _6322</t>
   </si>
   <si>
@@ -717,9 +720,6 @@
     <t>https://drive.google.com/file/d/1UGxYQjz06UbgdcJZw5Zn0lZ0a_AmTa0j/view</t>
   </si>
   <si>
-    <t>Evasion-Berck</t>
-  </si>
-  <si>
     <t>rotonde</t>
   </si>
   <si>
@@ -738,7 +738,10 @@
     <t>Oui (max 65°)</t>
   </si>
   <si>
-    <t>Rotonde-Berck</t>
+    <t>Patio23</t>
+  </si>
+  <si>
+    <t>23Patio23</t>
   </si>
   <si>
     <t>patio</t>
@@ -754,9 +757,6 @@
   </si>
   <si>
     <t>Oui (patio)</t>
-  </si>
-  <si>
-    <t>Patio-Berck</t>
   </si>
 </sst>
 </file>
@@ -1154,7 +1154,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A64D7D0E-AB10-4B85-8329-05C462C9F18A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A0AEDAF-E9C7-4DEC-BA1A-F1D2FA8D9543}">
   <dimension ref="A1:AR23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1566,8 +1566,8 @@
       <c r="AH3" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="AI3" s="2" t="s">
-        <v>76</v>
+      <c r="AI3" s="2">
+        <v>40803500</v>
       </c>
       <c r="AJ3" s="2">
         <v>15</v>
@@ -1576,7 +1576,7 @@
         <v>66</v>
       </c>
       <c r="AL3" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AM3" s="4" t="s">
         <v>67</v>
@@ -1602,13 +1602,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>79</v>
-      </c>
       <c r="D4" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>46</v>
@@ -1623,7 +1623,7 @@
         <v>49</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>51</v>
@@ -1638,7 +1638,7 @@
         <v>54</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O4" s="2" t="s">
         <v>56</v>
@@ -1698,10 +1698,10 @@
         <v>2</v>
       </c>
       <c r="AH4" s="2" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="AI4" s="2" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="AJ4" s="2">
         <v>15</v>
@@ -1736,13 +1736,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>46</v>
@@ -1757,13 +1757,13 @@
         <v>49</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>51</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>53</v>
@@ -1830,10 +1830,10 @@
         <v>2</v>
       </c>
       <c r="AH5" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="AI5" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="AJ5" s="2">
         <v>15</v>
@@ -1868,13 +1868,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>46</v>
@@ -1886,16 +1886,16 @@
         <v>48</v>
       </c>
       <c r="H6" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="K6" s="5" t="s">
         <v>92</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>95</v>
       </c>
       <c r="L6" s="3" t="s">
         <v>53</v>
@@ -1908,10 +1908,10 @@
         <v>56</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="R6" s="2" t="s">
         <v>59</v>
@@ -1961,11 +1961,11 @@
       <c r="AG6" s="2">
         <v>2</v>
       </c>
-      <c r="AH6" s="2" t="s">
-        <v>98</v>
+      <c r="AH6" s="5" t="s">
+        <v>95</v>
       </c>
       <c r="AI6" s="2" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="AJ6" s="2">
         <v>15</v>
@@ -2000,43 +2000,43 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>103</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>48</v>
       </c>
       <c r="H7" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="J7" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="K7" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="L7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="M7" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="N7" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="N7" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="O7" s="2" t="s">
         <v>56</v>
@@ -2045,7 +2045,7 @@
         <v>57</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="R7" s="2" t="s">
         <v>59</v>
@@ -2075,7 +2075,7 @@
         <v>60</v>
       </c>
       <c r="AA7" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AB7" s="3" t="s">
         <v>53</v>
@@ -2096,10 +2096,10 @@
         <v>1</v>
       </c>
       <c r="AH7" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="AI7" s="2" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="AJ7" s="2">
         <v>20</v>
@@ -2120,7 +2120,7 @@
         <v>53</v>
       </c>
       <c r="AP7" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AQ7" s="2" t="s">
         <v>69</v>
@@ -2134,19 +2134,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>115</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>48</v>
@@ -2155,13 +2155,13 @@
         <v>49</v>
       </c>
       <c r="I8" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="J8" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="J8" s="2" t="s">
-        <v>117</v>
-      </c>
       <c r="K8" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="L8" s="3" t="s">
         <v>53</v>
@@ -2207,7 +2207,7 @@
         <v>60</v>
       </c>
       <c r="AA8" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AB8" s="4" t="s">
         <v>60</v>
@@ -2228,10 +2228,10 @@
         <v>1</v>
       </c>
       <c r="AH8" s="2" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="AI8" s="2" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="AJ8" s="2">
         <v>20</v>
@@ -2252,7 +2252,7 @@
         <v>53</v>
       </c>
       <c r="AP8" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AQ8" s="2" t="s">
         <v>69</v>
@@ -2266,34 +2266,34 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="F9" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="I9" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="J9" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>124</v>
-      </c>
       <c r="K9" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>53</v>
@@ -2309,7 +2309,7 @@
         <v>57</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="R9" s="2" t="s">
         <v>59</v>
@@ -2360,10 +2360,10 @@
         <v>1</v>
       </c>
       <c r="AH9" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="AI9" s="2" t="s">
-        <v>88</v>
+        <v>124</v>
       </c>
       <c r="AJ9" s="2">
         <v>15</v>
@@ -2378,13 +2378,13 @@
         <v>67</v>
       </c>
       <c r="AN9" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="AO9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP9" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="AO9" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP9" s="2" t="s">
-        <v>127</v>
       </c>
       <c r="AQ9" s="2" t="s">
         <v>69</v>
@@ -2398,34 +2398,34 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H10" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="H10" s="2" t="s">
+      <c r="I10" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="J10" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="J10" s="2" t="s">
-        <v>134</v>
-      </c>
       <c r="K10" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="L10" s="3" t="s">
         <v>53</v>
@@ -2434,7 +2434,7 @@
         <v>54</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="O10" s="2" t="s">
         <v>56</v>
@@ -2446,7 +2446,7 @@
         <v>58</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="S10" s="4" t="s">
         <v>60</v>
@@ -2494,10 +2494,10 @@
         <v>1</v>
       </c>
       <c r="AH10" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AI10" s="2" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="AJ10" s="2">
         <v>15</v>
@@ -2518,7 +2518,7 @@
         <v>53</v>
       </c>
       <c r="AP10" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AQ10" s="2" t="s">
         <v>69</v>
@@ -2532,31 +2532,31 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>141</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>142</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>49</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>52</v>
@@ -2575,7 +2575,7 @@
         <v>57</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="R11" s="2" t="s">
         <v>59</v>
@@ -2611,7 +2611,7 @@
         <v>53</v>
       </c>
       <c r="AC11" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="AD11" s="3" t="s">
         <v>53</v>
@@ -2626,10 +2626,10 @@
         <v>1</v>
       </c>
       <c r="AH11" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="AI11" s="2" t="s">
         <v>144</v>
-      </c>
-      <c r="AI11" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="AJ11" s="2">
         <v>15</v>
@@ -2644,13 +2644,13 @@
         <v>67</v>
       </c>
       <c r="AN11" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="AO11" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP11" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="AO11" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP11" s="2" t="s">
-        <v>127</v>
       </c>
       <c r="AQ11" s="2" t="s">
         <v>69</v>
@@ -2679,7 +2679,7 @@
         <v>146</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>49</v>
@@ -2762,8 +2762,8 @@
       <c r="AH12" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="AI12" s="2" t="s">
-        <v>88</v>
+      <c r="AI12" s="2">
+        <v>74817733</v>
       </c>
       <c r="AJ12" s="2">
         <v>15</v>
@@ -2784,7 +2784,7 @@
         <v>53</v>
       </c>
       <c r="AP12" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AQ12" s="2" t="s">
         <v>154</v>
@@ -2813,16 +2813,16 @@
         <v>159</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>160</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>161</v>
@@ -2918,7 +2918,7 @@
         <v>53</v>
       </c>
       <c r="AP13" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AQ13" s="2" t="s">
         <v>154</v>
@@ -2947,19 +2947,19 @@
         <v>159</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>171</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="L14" s="4" t="s">
         <v>60</v>
@@ -2975,7 +2975,7 @@
         <v>57</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="R14" s="2" t="s">
         <v>59</v>
@@ -3028,8 +3028,8 @@
       <c r="AH14" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="AI14" s="2" t="s">
-        <v>88</v>
+      <c r="AI14" s="2">
+        <v>15246653</v>
       </c>
       <c r="AJ14" s="2">
         <v>20</v>
@@ -3050,7 +3050,7 @@
         <v>53</v>
       </c>
       <c r="AP14" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AQ14" s="2" t="s">
         <v>154</v>
@@ -3079,10 +3079,10 @@
         <v>159</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>179</v>
@@ -3091,7 +3091,7 @@
         <v>180</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>53</v>
@@ -3107,10 +3107,10 @@
         <v>57</v>
       </c>
       <c r="Q15" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="R15" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="S15" s="4" t="s">
         <v>60</v>
@@ -3160,8 +3160,8 @@
       <c r="AH15" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="AI15" s="2" t="s">
-        <v>88</v>
+      <c r="AI15" s="2">
+        <v>82562328</v>
       </c>
       <c r="AJ15" s="2">
         <v>20</v>
@@ -3182,7 +3182,7 @@
         <v>53</v>
       </c>
       <c r="AP15" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AQ15" s="2" t="s">
         <v>183</v>
@@ -3211,25 +3211,25 @@
         <v>159</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>187</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="L16" s="4" t="s">
         <v>60</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2" t="s">
@@ -3257,16 +3257,16 @@
         <v>62</v>
       </c>
       <c r="W16" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="X16" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="Y16" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="Z16" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="AA16" s="3" t="s">
         <v>53</v>
@@ -3275,7 +3275,7 @@
         <v>53</v>
       </c>
       <c r="AC16" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="AD16" s="3" t="s">
         <v>53</v>
@@ -3290,10 +3290,10 @@
         <v>1</v>
       </c>
       <c r="AH16" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="AI16" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="AJ16" s="2">
         <v>20</v>
@@ -3314,7 +3314,7 @@
         <v>53</v>
       </c>
       <c r="AP16" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AQ16" s="2" t="s">
         <v>154</v>
@@ -3343,7 +3343,7 @@
         <v>189</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>49</v>
@@ -3426,8 +3426,8 @@
       <c r="AH17" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="AI17" s="2" t="s">
-        <v>88</v>
+      <c r="AI17" s="2">
+        <v>66436003</v>
       </c>
       <c r="AJ17" s="2">
         <v>15</v>
@@ -3448,7 +3448,7 @@
         <v>53</v>
       </c>
       <c r="AP17" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AQ17" s="2" t="s">
         <v>154</v>
@@ -3477,10 +3477,10 @@
         <v>200</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>201</v>
@@ -3510,7 +3510,7 @@
         <v>204</v>
       </c>
       <c r="R18" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="S18" s="4" t="s">
         <v>60</v>
@@ -3561,7 +3561,7 @@
         <v>206</v>
       </c>
       <c r="AI18" s="2" t="s">
-        <v>88</v>
+        <v>207</v>
       </c>
       <c r="AJ18" s="2">
         <v>20</v>
@@ -3582,7 +3582,7 @@
         <v>53</v>
       </c>
       <c r="AP18" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AQ18" s="2" t="s">
         <v>154</v>
@@ -3596,13 +3596,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>199</v>
@@ -3611,13 +3611,13 @@
         <v>200</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>202</v>
@@ -3642,7 +3642,7 @@
         <v>58</v>
       </c>
       <c r="R19" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="S19" s="4" t="s">
         <v>60</v>
@@ -3690,10 +3690,10 @@
         <v>1</v>
       </c>
       <c r="AH19" s="2" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="AI19" s="2" t="s">
-        <v>88</v>
+        <v>207</v>
       </c>
       <c r="AJ19" s="2">
         <v>20</v>
@@ -3714,7 +3714,7 @@
         <v>53</v>
       </c>
       <c r="AP19" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AQ19" s="2" t="s">
         <v>154</v>
@@ -3773,7 +3773,7 @@
         <v>222</v>
       </c>
       <c r="Q20" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="R20" s="2" t="s">
         <v>59</v>
@@ -3818,13 +3818,13 @@
         <v>53</v>
       </c>
       <c r="AF20" s="2" t="s">
-        <v>63</v>
+        <v>223</v>
       </c>
       <c r="AG20" s="2">
         <v>1</v>
       </c>
       <c r="AH20" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="AI20" s="2">
         <v>83968280</v>
@@ -3848,7 +3848,7 @@
         <v>53</v>
       </c>
       <c r="AP20" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AQ20" s="2" t="s">
         <v>154</v>
@@ -3862,16 +3862,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>216</v>
@@ -3889,7 +3889,7 @@
         <v>218</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="L21" s="3" t="s">
         <v>53</v>
@@ -3898,7 +3898,7 @@
         <v>220</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="O21" s="2" t="s">
         <v>56</v>
@@ -3937,7 +3937,7 @@
         <v>60</v>
       </c>
       <c r="AA21" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AB21" s="4" t="s">
         <v>60</v>
@@ -3952,16 +3952,16 @@
         <v>53</v>
       </c>
       <c r="AF21" s="2" t="s">
-        <v>63</v>
+        <v>223</v>
       </c>
       <c r="AG21" s="2">
         <v>1</v>
       </c>
       <c r="AH21" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="AI21" s="2" t="s">
-        <v>88</v>
+        <v>224</v>
+      </c>
+      <c r="AI21" s="2">
+        <v>83968280</v>
       </c>
       <c r="AJ21" s="2">
         <v>20</v>
@@ -3982,7 +3982,7 @@
         <v>53</v>
       </c>
       <c r="AP21" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AQ21" s="2" t="s">
         <v>154</v>
@@ -4005,7 +4005,7 @@
         <v>232</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>216</v>
@@ -4014,7 +4014,7 @@
         <v>212</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>233</v>
@@ -4023,7 +4023,7 @@
         <v>234</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="L22" s="3" t="s">
         <v>53</v>
@@ -4069,7 +4069,7 @@
         <v>60</v>
       </c>
       <c r="AA22" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AB22" s="4" t="s">
         <v>235</v>
@@ -4093,7 +4093,7 @@
         <v>236</v>
       </c>
       <c r="AI22" s="2" t="s">
-        <v>88</v>
+        <v>237</v>
       </c>
       <c r="AJ22" s="2">
         <v>20</v>
@@ -4114,7 +4114,7 @@
         <v>53</v>
       </c>
       <c r="AP22" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AQ22" s="2" t="s">
         <v>154</v>
@@ -4128,16 +4128,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>216</v>
@@ -4152,10 +4152,10 @@
         <v>179</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="L23" s="3" t="s">
         <v>53</v>
@@ -4164,7 +4164,7 @@
         <v>220</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="O23" s="2" t="s">
         <v>56</v>
@@ -4203,13 +4203,13 @@
         <v>60</v>
       </c>
       <c r="AA23" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="AB23" s="3" t="s">
         <v>53</v>
       </c>
       <c r="AC23" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="AD23" s="4" t="s">
         <v>60</v>
@@ -4224,10 +4224,10 @@
         <v>1</v>
       </c>
       <c r="AH23" s="2" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="AI23" s="2" t="s">
-        <v>88</v>
+        <v>237</v>
       </c>
       <c r="AJ23" s="2">
         <v>20</v>
@@ -4248,7 +4248,7 @@
         <v>53</v>
       </c>
       <c r="AP23" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AQ23" s="2" t="s">
         <v>154</v>
@@ -4258,7 +4258,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AR23" xr:uid="{A64D7D0E-AB10-4B85-8329-05C462C9F18A}"/>
+  <autoFilter ref="A1:AR23" xr:uid="{8A0AEDAF-E9C7-4DEC-BA1A-F1D2FA8D9543}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>